<commit_message>
Add wall-run-up and sprint window vault
</commit_message>
<xml_diff>
--- a/Parkour/SourseFiles/Info.xlsx
+++ b/Parkour/SourseFiles/Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Zomboid\Workshop\Parkour\SourseFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764BDEF9-5203-4809-A3CF-0623ED164F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C398A73-6869-4313-B08F-9B7B2516AA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="2385" windowWidth="33525" windowHeight="14355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="645" yWindow="5385" windowWidth="33525" windowHeight="14355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>2.533 sec / SpeedScale 1.50 × TimePc 0.95 ≈ 1.604 sec</t>
   </si>
@@ -79,6 +79,18 @@
       </rPr>
       <t xml:space="preserve">. </t>
     </r>
+  </si>
+  <si>
+    <t>добавить анимку на перелаз окна</t>
+  </si>
+  <si>
+    <t>Добавить анимку для высокого забора</t>
+  </si>
+  <si>
+    <t>Добавить Урон на волт через окно</t>
+  </si>
+  <si>
+    <t>Добавить анимку простого перелаза</t>
   </si>
 </sst>
 </file>
@@ -407,20 +419,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:B4"/>
+  <dimension ref="B2:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="51.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:5">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="2:2" ht="60">
+    <row r="3" spans="2:5">
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="60">
       <c r="B4" s="2" t="s">
         <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="E5" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>